<commit_message>
Local updates: data files + pipeline fixes
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D121"/>
+  <dimension ref="A1:D131"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2093,9 +2093,149 @@
         <v>0</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>05/01</v>
+      </c>
+      <c r="B122">
+        <v>25</v>
+      </c>
+      <c r="C122">
+        <v>3</v>
+      </c>
+      <c r="D122">
+        <v>936.5</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>05/02</v>
+      </c>
+      <c r="B123">
+        <v>25</v>
+      </c>
+      <c r="C123">
+        <v>3</v>
+      </c>
+      <c r="D123">
+        <v>893.7</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>05/03</v>
+      </c>
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124">
+        <v>0</v>
+      </c>
+      <c r="D124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>05/04</v>
+      </c>
+      <c r="B125">
+        <v>8.33</v>
+      </c>
+      <c r="C125">
+        <v>1</v>
+      </c>
+      <c r="D125">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>05/05</v>
+      </c>
+      <c r="B126">
+        <v>0</v>
+      </c>
+      <c r="C126">
+        <v>0</v>
+      </c>
+      <c r="D126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>05/06</v>
+      </c>
+      <c r="B127">
+        <v>0</v>
+      </c>
+      <c r="C127">
+        <v>0</v>
+      </c>
+      <c r="D127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>05/07</v>
+      </c>
+      <c r="B128">
+        <v>0</v>
+      </c>
+      <c r="C128">
+        <v>0</v>
+      </c>
+      <c r="D128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>05/08</v>
+      </c>
+      <c r="B129">
+        <v>41.67</v>
+      </c>
+      <c r="C129">
+        <v>5</v>
+      </c>
+      <c r="D129">
+        <v>1715</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>05/09</v>
+      </c>
+      <c r="B130">
+        <v>41.67</v>
+      </c>
+      <c r="C130">
+        <v>5</v>
+      </c>
+      <c r="D130">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>05/10</v>
+      </c>
+      <c r="B131">
+        <v>0</v>
+      </c>
+      <c r="C131">
+        <v>0</v>
+      </c>
+      <c r="D131">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D121"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D131"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revamp Monday Slack digest: pickup, forward pace, weekend watch
Replaces YTD-focused digest with pickup (vs last week's snapshot),
a 5-week forward pace table against seasonal targets, weekend watch,
and a single AI-generated action item. Adapts Cloudbeds export format
change (ADR/Room Rates columns). Weekly data update for Jun 15.
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D152"/>
+  <dimension ref="A1:D166"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1510,13 +1510,13 @@
         <v>03/20</v>
       </c>
       <c r="B80">
-        <v>250.45454545454547</v>
+        <v>243.76</v>
       </c>
       <c r="C80">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D80">
-        <v>2755</v>
+        <v>2437.6</v>
       </c>
     </row>
     <row r="81">
@@ -1524,13 +1524,13 @@
         <v>03/21</v>
       </c>
       <c r="B81">
-        <v>236.6</v>
+        <v>227.6222222222222</v>
       </c>
       <c r="C81">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D81">
-        <v>2366</v>
+        <v>2048.6</v>
       </c>
     </row>
     <row r="82">
@@ -2350,13 +2350,13 @@
         <v>05/19</v>
       </c>
       <c r="B140">
-        <v>200.7166666666667</v>
+        <v>200.71666666666667</v>
       </c>
       <c r="C140">
         <v>6</v>
       </c>
       <c r="D140">
-        <v>1204.3000000000002</v>
+        <v>1204.3</v>
       </c>
     </row>
     <row r="141">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.2125</v>
+        <v>256.21250000000003</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.5499999999997</v>
+        <v>3074.55</v>
       </c>
     </row>
     <row r="145">
@@ -2426,7 +2426,7 @@
         <v>10</v>
       </c>
       <c r="D145">
-        <v>2962.4500000000003</v>
+        <v>2962.45</v>
       </c>
     </row>
     <row r="146">
@@ -2504,13 +2504,13 @@
         <v>05/30</v>
       </c>
       <c r="B151">
-        <v>274.58000000000004</v>
+        <v>274.58</v>
       </c>
       <c r="C151">
         <v>5</v>
       </c>
       <c r="D151">
-        <v>1372.9</v>
+        <v>1372.8999999999999</v>
       </c>
     </row>
     <row r="152">
@@ -2527,9 +2527,205 @@
         <v>476.75</v>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>06/01</v>
+      </c>
+      <c r="B153">
+        <v>177.825</v>
+      </c>
+      <c r="C153">
+        <v>2</v>
+      </c>
+      <c r="D153">
+        <v>355.65</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>06/02</v>
+      </c>
+      <c r="B154">
+        <v>215.05</v>
+      </c>
+      <c r="C154">
+        <v>2</v>
+      </c>
+      <c r="D154">
+        <v>430.1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>06/03</v>
+      </c>
+      <c r="B155">
+        <v>215.05</v>
+      </c>
+      <c r="C155">
+        <v>2</v>
+      </c>
+      <c r="D155">
+        <v>430.1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>06/04</v>
+      </c>
+      <c r="B156">
+        <v>206.1</v>
+      </c>
+      <c r="C156">
+        <v>1</v>
+      </c>
+      <c r="D156">
+        <v>206.1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>06/05</v>
+      </c>
+      <c r="B157">
+        <v>258.96666666666664</v>
+      </c>
+      <c r="C157">
+        <v>3</v>
+      </c>
+      <c r="D157">
+        <v>776.9</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>06/06</v>
+      </c>
+      <c r="B158">
+        <v>276.152</v>
+      </c>
+      <c r="C158">
+        <v>5</v>
+      </c>
+      <c r="D158">
+        <v>1380.76</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>06/07</v>
+      </c>
+      <c r="B159">
+        <v>248.71428571428572</v>
+      </c>
+      <c r="C159">
+        <v>7</v>
+      </c>
+      <c r="D159">
+        <v>1741</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>06/08</v>
+      </c>
+      <c r="B160">
+        <v>0</v>
+      </c>
+      <c r="C160">
+        <v>2</v>
+      </c>
+      <c r="D160">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>06/09</v>
+      </c>
+      <c r="B161">
+        <v>86.72999999999999</v>
+      </c>
+      <c r="C161">
+        <v>5</v>
+      </c>
+      <c r="D161">
+        <v>433.65</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>06/10</v>
+      </c>
+      <c r="B162">
+        <v>119.5</v>
+      </c>
+      <c r="C162">
+        <v>2</v>
+      </c>
+      <c r="D162">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>06/11</v>
+      </c>
+      <c r="B163">
+        <v>237.04999999999998</v>
+      </c>
+      <c r="C163">
+        <v>6</v>
+      </c>
+      <c r="D163">
+        <v>1422.3</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>06/12</v>
+      </c>
+      <c r="B164">
+        <v>250.42374999999998</v>
+      </c>
+      <c r="C164">
+        <v>8</v>
+      </c>
+      <c r="D164">
+        <v>2003.3899999999999</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>06/13</v>
+      </c>
+      <c r="B165">
+        <v>245.79777777777775</v>
+      </c>
+      <c r="C165">
+        <v>9</v>
+      </c>
+      <c r="D165">
+        <v>2212.18</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>06/14</v>
+      </c>
+      <c r="B166">
+        <v>225.42500000000004</v>
+      </c>
+      <c r="C166">
+        <v>6</v>
+      </c>
+      <c r="D166">
+        <v>1352.5500000000002</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D152"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D166"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Jun 22 Cloudbeds export (YTD + pace) — previous data was stale Jun 15
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D166"/>
+  <dimension ref="A1:D173"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2350,13 +2350,13 @@
         <v>05/19</v>
       </c>
       <c r="B140">
-        <v>200.71666666666667</v>
+        <v>200.7166666666667</v>
       </c>
       <c r="C140">
         <v>6</v>
       </c>
       <c r="D140">
-        <v>1204.3</v>
+        <v>1204.3000000000002</v>
       </c>
     </row>
     <row r="141">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.21250000000003</v>
+        <v>256.2125</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.55</v>
+        <v>3074.5499999999997</v>
       </c>
     </row>
     <row r="145">
@@ -2504,13 +2504,13 @@
         <v>05/30</v>
       </c>
       <c r="B151">
-        <v>274.58</v>
+        <v>274.58000000000004</v>
       </c>
       <c r="C151">
         <v>5</v>
       </c>
       <c r="D151">
-        <v>1372.8999999999999</v>
+        <v>1372.9</v>
       </c>
     </row>
     <row r="152">
@@ -2672,13 +2672,13 @@
         <v>06/11</v>
       </c>
       <c r="B163">
-        <v>237.04999999999998</v>
+        <v>237.05000000000004</v>
       </c>
       <c r="C163">
         <v>6</v>
       </c>
       <c r="D163">
-        <v>1422.3</v>
+        <v>1422.3000000000002</v>
       </c>
     </row>
     <row r="164">
@@ -2714,18 +2714,116 @@
         <v>06/14</v>
       </c>
       <c r="B166">
-        <v>225.42500000000004</v>
+        <v>225.42499999999998</v>
       </c>
       <c r="C166">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>1352.5500000000002</v>
+        <v>1352.55</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>06/15</v>
+      </c>
+      <c r="B167">
+        <v>205.05</v>
+      </c>
+      <c r="C167">
+        <v>4</v>
+      </c>
+      <c r="D167">
+        <v>820.2</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>06/16</v>
+      </c>
+      <c r="B168">
+        <v>199.76999999999998</v>
+      </c>
+      <c r="C168">
+        <v>6</v>
+      </c>
+      <c r="D168">
+        <v>1198.62</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>06/17</v>
+      </c>
+      <c r="B169">
+        <v>212.05666666666667</v>
+      </c>
+      <c r="C169">
+        <v>9</v>
+      </c>
+      <c r="D169">
+        <v>1908.51</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>06/18</v>
+      </c>
+      <c r="B170">
+        <v>247.25</v>
+      </c>
+      <c r="C170">
+        <v>4</v>
+      </c>
+      <c r="D170">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>06/19</v>
+      </c>
+      <c r="B171">
+        <v>274.144</v>
+      </c>
+      <c r="C171">
+        <v>10</v>
+      </c>
+      <c r="D171">
+        <v>2741.44</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>06/20</v>
+      </c>
+      <c r="B172">
+        <v>300.1233333333333</v>
+      </c>
+      <c r="C172">
+        <v>9</v>
+      </c>
+      <c r="D172">
+        <v>2701.1099999999997</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>06/21</v>
+      </c>
+      <c r="B173">
+        <v>240.55714285714288</v>
+      </c>
+      <c r="C173">
+        <v>7</v>
+      </c>
+      <c r="D173">
+        <v>1683.9</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D166"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D173"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-06-29
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D173"/>
+  <dimension ref="A1:D180"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2392,13 +2392,13 @@
         <v>05/22</v>
       </c>
       <c r="B143">
-        <v>278.4944444444444</v>
+        <v>278.49444444444447</v>
       </c>
       <c r="C143">
         <v>9</v>
       </c>
       <c r="D143">
-        <v>2506.45</v>
+        <v>2506.4500000000003</v>
       </c>
     </row>
     <row r="144">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.2125</v>
+        <v>256.21250000000003</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.5499999999997</v>
+        <v>3074.55</v>
       </c>
     </row>
     <row r="145">
@@ -2672,13 +2672,13 @@
         <v>06/11</v>
       </c>
       <c r="B163">
-        <v>237.05000000000004</v>
+        <v>237.04999999999998</v>
       </c>
       <c r="C163">
         <v>6</v>
       </c>
       <c r="D163">
-        <v>1422.3000000000002</v>
+        <v>1422.3</v>
       </c>
     </row>
     <row r="164">
@@ -2784,13 +2784,13 @@
         <v>06/19</v>
       </c>
       <c r="B171">
-        <v>274.144</v>
+        <v>274.14399999999995</v>
       </c>
       <c r="C171">
         <v>10</v>
       </c>
       <c r="D171">
-        <v>2741.44</v>
+        <v>2741.4399999999996</v>
       </c>
     </row>
     <row r="172">
@@ -2812,18 +2812,116 @@
         <v>06/21</v>
       </c>
       <c r="B173">
-        <v>240.55714285714288</v>
+        <v>240.55714285714285</v>
       </c>
       <c r="C173">
         <v>7</v>
       </c>
       <c r="D173">
-        <v>1683.9</v>
+        <v>1683.8999999999999</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>06/22</v>
+      </c>
+      <c r="B174">
+        <v>220.18</v>
+      </c>
+      <c r="C174">
+        <v>5</v>
+      </c>
+      <c r="D174">
+        <v>1100.9</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>06/23</v>
+      </c>
+      <c r="B175">
+        <v>207.88333333333333</v>
+      </c>
+      <c r="C175">
+        <v>6</v>
+      </c>
+      <c r="D175">
+        <v>1247.3</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>06/24</v>
+      </c>
+      <c r="B176">
+        <v>185.91666666666666</v>
+      </c>
+      <c r="C176">
+        <v>6</v>
+      </c>
+      <c r="D176">
+        <v>1115.5</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>06/25</v>
+      </c>
+      <c r="B177">
+        <v>322</v>
+      </c>
+      <c r="C177">
+        <v>1</v>
+      </c>
+      <c r="D177">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>06/26</v>
+      </c>
+      <c r="B178">
+        <v>257.8111111111111</v>
+      </c>
+      <c r="C178">
+        <v>9</v>
+      </c>
+      <c r="D178">
+        <v>2320.2999999999997</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>06/27</v>
+      </c>
+      <c r="B179">
+        <v>251.96545454545458</v>
+      </c>
+      <c r="C179">
+        <v>11</v>
+      </c>
+      <c r="D179">
+        <v>2771.6200000000003</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>06/28</v>
+      </c>
+      <c r="B180">
+        <v>235.01666666666665</v>
+      </c>
+      <c r="C180">
+        <v>6</v>
+      </c>
+      <c r="D180">
+        <v>1410.1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D173"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D180"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-07-06
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D180"/>
+  <dimension ref="A1:D187"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2392,13 +2392,13 @@
         <v>05/22</v>
       </c>
       <c r="B143">
-        <v>278.49444444444447</v>
+        <v>278.4944444444444</v>
       </c>
       <c r="C143">
         <v>9</v>
       </c>
       <c r="D143">
-        <v>2506.4500000000003</v>
+        <v>2506.45</v>
       </c>
     </row>
     <row r="144">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.21250000000003</v>
+        <v>256.2125</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.55</v>
+        <v>3074.5499999999997</v>
       </c>
     </row>
     <row r="145">
@@ -2714,13 +2714,13 @@
         <v>06/14</v>
       </c>
       <c r="B166">
-        <v>225.42499999999998</v>
+        <v>225.42500000000004</v>
       </c>
       <c r="C166">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>1352.55</v>
+        <v>1352.5500000000002</v>
       </c>
     </row>
     <row r="167">
@@ -2784,13 +2784,13 @@
         <v>06/19</v>
       </c>
       <c r="B171">
-        <v>274.14399999999995</v>
+        <v>274.144</v>
       </c>
       <c r="C171">
         <v>10</v>
       </c>
       <c r="D171">
-        <v>2741.4399999999996</v>
+        <v>2741.44</v>
       </c>
     </row>
     <row r="172">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>257.8111111111111</v>
+        <v>257.81111111111113</v>
       </c>
       <c r="C178">
         <v>9</v>
       </c>
       <c r="D178">
-        <v>2320.2999999999997</v>
+        <v>2320.3</v>
       </c>
     </row>
     <row r="179">
@@ -2896,13 +2896,13 @@
         <v>06/27</v>
       </c>
       <c r="B179">
-        <v>251.96545454545458</v>
+        <v>251.96545454545455</v>
       </c>
       <c r="C179">
         <v>11</v>
       </c>
       <c r="D179">
-        <v>2771.6200000000003</v>
+        <v>2771.62</v>
       </c>
     </row>
     <row r="180">
@@ -2919,9 +2919,107 @@
         <v>1410.1</v>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>06/29</v>
+      </c>
+      <c r="B181">
+        <v>243.275</v>
+      </c>
+      <c r="C181">
+        <v>4</v>
+      </c>
+      <c r="D181">
+        <v>973.1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>06/30</v>
+      </c>
+      <c r="B182">
+        <v>251.025</v>
+      </c>
+      <c r="C182">
+        <v>4</v>
+      </c>
+      <c r="D182">
+        <v>1004.1</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>07/01</v>
+      </c>
+      <c r="B183">
+        <v>299</v>
+      </c>
+      <c r="C183">
+        <v>1</v>
+      </c>
+      <c r="D183">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>07/02</v>
+      </c>
+      <c r="B184">
+        <v>298</v>
+      </c>
+      <c r="C184">
+        <v>7</v>
+      </c>
+      <c r="D184">
+        <v>2086</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>07/03</v>
+      </c>
+      <c r="B185">
+        <v>305.1666666666667</v>
+      </c>
+      <c r="C185">
+        <v>12</v>
+      </c>
+      <c r="D185">
+        <v>3662</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>07/04</v>
+      </c>
+      <c r="B186">
+        <v>318.6333333333333</v>
+      </c>
+      <c r="C186">
+        <v>12</v>
+      </c>
+      <c r="D186">
+        <v>3823.6</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>07/05</v>
+      </c>
+      <c r="B187">
+        <v>233.66666666666666</v>
+      </c>
+      <c r="C187">
+        <v>3</v>
+      </c>
+      <c r="D187">
+        <v>701</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D180"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D187"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-07-13
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D187"/>
+  <dimension ref="A1:D194"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2350,13 +2350,13 @@
         <v>05/19</v>
       </c>
       <c r="B140">
-        <v>200.7166666666667</v>
+        <v>200.71666666666667</v>
       </c>
       <c r="C140">
         <v>6</v>
       </c>
       <c r="D140">
-        <v>1204.3000000000002</v>
+        <v>1204.3</v>
       </c>
     </row>
     <row r="141">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.2125</v>
+        <v>256.21250000000003</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.5499999999997</v>
+        <v>3074.55</v>
       </c>
     </row>
     <row r="145">
@@ -2448,13 +2448,13 @@
         <v>05/26</v>
       </c>
       <c r="B147">
-        <v>190.15555555555554</v>
+        <v>190.15555555555557</v>
       </c>
       <c r="C147">
         <v>9</v>
       </c>
       <c r="D147">
-        <v>1711.3999999999999</v>
+        <v>1711.4</v>
       </c>
     </row>
     <row r="148">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>245.79777777777775</v>
+        <v>245.7977777777778</v>
       </c>
       <c r="C165">
         <v>9</v>
       </c>
       <c r="D165">
-        <v>2212.18</v>
+        <v>2212.1800000000003</v>
       </c>
     </row>
     <row r="166">
@@ -2714,13 +2714,13 @@
         <v>06/14</v>
       </c>
       <c r="B166">
-        <v>225.42500000000004</v>
+        <v>225.42499999999998</v>
       </c>
       <c r="C166">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>1352.5500000000002</v>
+        <v>1352.55</v>
       </c>
     </row>
     <row r="167">
@@ -2812,13 +2812,13 @@
         <v>06/21</v>
       </c>
       <c r="B173">
-        <v>240.55714285714285</v>
+        <v>240.55714285714288</v>
       </c>
       <c r="C173">
         <v>7</v>
       </c>
       <c r="D173">
-        <v>1683.8999999999999</v>
+        <v>1683.9</v>
       </c>
     </row>
     <row r="174">
@@ -3017,9 +3017,107 @@
         <v>701</v>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>07/06</v>
+      </c>
+      <c r="B188">
+        <v>245.66666666666666</v>
+      </c>
+      <c r="C188">
+        <v>3</v>
+      </c>
+      <c r="D188">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>07/07</v>
+      </c>
+      <c r="B189">
+        <v>239</v>
+      </c>
+      <c r="C189">
+        <v>2</v>
+      </c>
+      <c r="D189">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>07/08</v>
+      </c>
+      <c r="B190">
+        <v>261.5</v>
+      </c>
+      <c r="C190">
+        <v>2</v>
+      </c>
+      <c r="D190">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>07/09</v>
+      </c>
+      <c r="B191">
+        <v>297</v>
+      </c>
+      <c r="C191">
+        <v>2</v>
+      </c>
+      <c r="D191">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>07/10</v>
+      </c>
+      <c r="B192">
+        <v>317.1272727272727</v>
+      </c>
+      <c r="C192">
+        <v>11</v>
+      </c>
+      <c r="D192">
+        <v>3488.4</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>07/11</v>
+      </c>
+      <c r="B193">
+        <v>308.14166666666665</v>
+      </c>
+      <c r="C193">
+        <v>12</v>
+      </c>
+      <c r="D193">
+        <v>3697.7</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>07/12</v>
+      </c>
+      <c r="B194">
+        <v>216.72727272727272</v>
+      </c>
+      <c r="C194">
+        <v>11</v>
+      </c>
+      <c r="D194">
+        <v>2384</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D187"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D194"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-07-20
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D194"/>
+  <dimension ref="A1:D201"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1034,13 +1034,13 @@
         <v>02/14</v>
       </c>
       <c r="B46">
-        <v>202.01600000000002</v>
+        <v>202.016</v>
       </c>
       <c r="C46">
         <v>5</v>
       </c>
       <c r="D46">
-        <v>1010.08</v>
+        <v>1010.0799999999999</v>
       </c>
     </row>
     <row r="47">
@@ -2350,13 +2350,13 @@
         <v>05/19</v>
       </c>
       <c r="B140">
-        <v>200.71666666666667</v>
+        <v>200.7166666666667</v>
       </c>
       <c r="C140">
         <v>6</v>
       </c>
       <c r="D140">
-        <v>1204.3</v>
+        <v>1204.3000000000002</v>
       </c>
     </row>
     <row r="141">
@@ -2448,13 +2448,13 @@
         <v>05/26</v>
       </c>
       <c r="B147">
-        <v>190.15555555555557</v>
+        <v>190.15555555555554</v>
       </c>
       <c r="C147">
         <v>9</v>
       </c>
       <c r="D147">
-        <v>1711.4</v>
+        <v>1711.3999999999999</v>
       </c>
     </row>
     <row r="148">
@@ -2504,13 +2504,13 @@
         <v>05/30</v>
       </c>
       <c r="B151">
-        <v>274.58000000000004</v>
+        <v>274.58</v>
       </c>
       <c r="C151">
         <v>5</v>
       </c>
       <c r="D151">
-        <v>1372.9</v>
+        <v>1372.8999999999999</v>
       </c>
     </row>
     <row r="152">
@@ -2672,13 +2672,13 @@
         <v>06/11</v>
       </c>
       <c r="B163">
-        <v>237.04999999999998</v>
+        <v>237.05000000000004</v>
       </c>
       <c r="C163">
         <v>6</v>
       </c>
       <c r="D163">
-        <v>1422.3</v>
+        <v>1422.3000000000002</v>
       </c>
     </row>
     <row r="164">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>245.7977777777778</v>
+        <v>245.79777777777775</v>
       </c>
       <c r="C165">
         <v>9</v>
       </c>
       <c r="D165">
-        <v>2212.1800000000003</v>
+        <v>2212.18</v>
       </c>
     </row>
     <row r="166">
@@ -2784,13 +2784,13 @@
         <v>06/19</v>
       </c>
       <c r="B171">
-        <v>274.144</v>
+        <v>274.14399999999995</v>
       </c>
       <c r="C171">
         <v>10</v>
       </c>
       <c r="D171">
-        <v>2741.44</v>
+        <v>2741.4399999999996</v>
       </c>
     </row>
     <row r="172">
@@ -3115,9 +3115,107 @@
         <v>2384</v>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>07/13</v>
+      </c>
+      <c r="B195">
+        <v>195.10875</v>
+      </c>
+      <c r="C195">
+        <v>8</v>
+      </c>
+      <c r="D195">
+        <v>1560.87</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>07/14</v>
+      </c>
+      <c r="B196">
+        <v>214</v>
+      </c>
+      <c r="C196">
+        <v>2</v>
+      </c>
+      <c r="D196">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>07/15</v>
+      </c>
+      <c r="B197">
+        <v>244.5</v>
+      </c>
+      <c r="C197">
+        <v>2</v>
+      </c>
+      <c r="D197">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>07/16</v>
+      </c>
+      <c r="B198">
+        <v>221.2</v>
+      </c>
+      <c r="C198">
+        <v>5</v>
+      </c>
+      <c r="D198">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>07/17</v>
+      </c>
+      <c r="B199">
+        <v>322</v>
+      </c>
+      <c r="C199">
+        <v>9</v>
+      </c>
+      <c r="D199">
+        <v>2898</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>07/18</v>
+      </c>
+      <c r="B200">
+        <v>375.2</v>
+      </c>
+      <c r="C200">
+        <v>5</v>
+      </c>
+      <c r="D200">
+        <v>1876</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>07/19</v>
+      </c>
+      <c r="B201">
+        <v>165</v>
+      </c>
+      <c r="C201">
+        <v>1</v>
+      </c>
+      <c r="D201">
+        <v>165</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D194"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D201"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-07-27
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D201"/>
+  <dimension ref="A1:D208"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1034,13 +1034,13 @@
         <v>02/14</v>
       </c>
       <c r="B46">
-        <v>202.016</v>
+        <v>202.01600000000002</v>
       </c>
       <c r="C46">
         <v>5</v>
       </c>
       <c r="D46">
-        <v>1010.0799999999999</v>
+        <v>1010.08</v>
       </c>
     </row>
     <row r="47">
@@ -2350,13 +2350,13 @@
         <v>05/19</v>
       </c>
       <c r="B140">
-        <v>200.7166666666667</v>
+        <v>200.71666666666667</v>
       </c>
       <c r="C140">
         <v>6</v>
       </c>
       <c r="D140">
-        <v>1204.3000000000002</v>
+        <v>1204.3</v>
       </c>
     </row>
     <row r="141">
@@ -2392,13 +2392,13 @@
         <v>05/22</v>
       </c>
       <c r="B143">
-        <v>278.4944444444444</v>
+        <v>278.49444444444447</v>
       </c>
       <c r="C143">
         <v>9</v>
       </c>
       <c r="D143">
-        <v>2506.45</v>
+        <v>2506.4500000000003</v>
       </c>
     </row>
     <row r="144">
@@ -2448,13 +2448,13 @@
         <v>05/26</v>
       </c>
       <c r="B147">
-        <v>190.15555555555554</v>
+        <v>190.15555555555557</v>
       </c>
       <c r="C147">
         <v>9</v>
       </c>
       <c r="D147">
-        <v>1711.3999999999999</v>
+        <v>1711.4</v>
       </c>
     </row>
     <row r="148">
@@ -2504,13 +2504,13 @@
         <v>05/30</v>
       </c>
       <c r="B151">
-        <v>274.58</v>
+        <v>274.58000000000004</v>
       </c>
       <c r="C151">
         <v>5</v>
       </c>
       <c r="D151">
-        <v>1372.8999999999999</v>
+        <v>1372.9</v>
       </c>
     </row>
     <row r="152">
@@ -2672,13 +2672,13 @@
         <v>06/11</v>
       </c>
       <c r="B163">
-        <v>237.05000000000004</v>
+        <v>237.04999999999998</v>
       </c>
       <c r="C163">
         <v>6</v>
       </c>
       <c r="D163">
-        <v>1422.3000000000002</v>
+        <v>1422.3</v>
       </c>
     </row>
     <row r="164">
@@ -2798,13 +2798,13 @@
         <v>06/20</v>
       </c>
       <c r="B172">
-        <v>300.1233333333333</v>
+        <v>300.12333333333333</v>
       </c>
       <c r="C172">
         <v>9</v>
       </c>
       <c r="D172">
-        <v>2701.1099999999997</v>
+        <v>2701.11</v>
       </c>
     </row>
     <row r="173">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>257.81111111111113</v>
+        <v>257.8111111111111</v>
       </c>
       <c r="C178">
         <v>9</v>
       </c>
       <c r="D178">
-        <v>2320.3</v>
+        <v>2320.2999999999997</v>
       </c>
     </row>
     <row r="179">
@@ -2896,13 +2896,13 @@
         <v>06/27</v>
       </c>
       <c r="B179">
-        <v>251.96545454545455</v>
+        <v>251.9654545454545</v>
       </c>
       <c r="C179">
         <v>11</v>
       </c>
       <c r="D179">
-        <v>2771.62</v>
+        <v>2771.6199999999994</v>
       </c>
     </row>
     <row r="180">
@@ -3213,9 +3213,107 @@
         <v>165</v>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>07/20</v>
+      </c>
+      <c r="B202">
+        <v>166.62666666666667</v>
+      </c>
+      <c r="C202">
+        <v>3</v>
+      </c>
+      <c r="D202">
+        <v>499.88</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>07/21</v>
+      </c>
+      <c r="B203">
+        <v>169.42249999999999</v>
+      </c>
+      <c r="C203">
+        <v>4</v>
+      </c>
+      <c r="D203">
+        <v>677.6899999999999</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>07/22</v>
+      </c>
+      <c r="B204">
+        <v>191.25</v>
+      </c>
+      <c r="C204">
+        <v>3</v>
+      </c>
+      <c r="D204">
+        <v>573.75</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>07/23</v>
+      </c>
+      <c r="B205">
+        <v>241</v>
+      </c>
+      <c r="C205">
+        <v>4</v>
+      </c>
+      <c r="D205">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>07/24</v>
+      </c>
+      <c r="B206">
+        <v>272.64363636363635</v>
+      </c>
+      <c r="C206">
+        <v>11</v>
+      </c>
+      <c r="D206">
+        <v>2999.08</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>07/25</v>
+      </c>
+      <c r="B207">
+        <v>257.58</v>
+      </c>
+      <c r="C207">
+        <v>11</v>
+      </c>
+      <c r="D207">
+        <v>2833.38</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>07/26</v>
+      </c>
+      <c r="B208">
+        <v>237.82222222222222</v>
+      </c>
+      <c r="C208">
+        <v>9</v>
+      </c>
+      <c r="D208">
+        <v>2140.4</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D201"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D208"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-08-03
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D208"/>
+  <dimension ref="A1:D215"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1034,13 +1034,13 @@
         <v>02/14</v>
       </c>
       <c r="B46">
-        <v>202.01600000000002</v>
+        <v>202.016</v>
       </c>
       <c r="C46">
         <v>5</v>
       </c>
       <c r="D46">
-        <v>1010.08</v>
+        <v>1010.0799999999999</v>
       </c>
     </row>
     <row r="47">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.21250000000003</v>
+        <v>256.2125</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.55</v>
+        <v>3074.5499999999997</v>
       </c>
     </row>
     <row r="145">
@@ -2448,13 +2448,13 @@
         <v>05/26</v>
       </c>
       <c r="B147">
-        <v>190.15555555555557</v>
+        <v>190.15555555555554</v>
       </c>
       <c r="C147">
         <v>9</v>
       </c>
       <c r="D147">
-        <v>1711.4</v>
+        <v>1711.3999999999999</v>
       </c>
     </row>
     <row r="148">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>245.79777777777775</v>
+        <v>245.7977777777778</v>
       </c>
       <c r="C165">
         <v>9</v>
       </c>
       <c r="D165">
-        <v>2212.18</v>
+        <v>2212.1800000000003</v>
       </c>
     </row>
     <row r="166">
@@ -2784,13 +2784,13 @@
         <v>06/19</v>
       </c>
       <c r="B171">
-        <v>274.14399999999995</v>
+        <v>274.144</v>
       </c>
       <c r="C171">
         <v>10</v>
       </c>
       <c r="D171">
-        <v>2741.4399999999996</v>
+        <v>2741.44</v>
       </c>
     </row>
     <row r="172">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>257.8111111111111</v>
+        <v>257.81111111111113</v>
       </c>
       <c r="C178">
         <v>9</v>
       </c>
       <c r="D178">
-        <v>2320.2999999999997</v>
+        <v>2320.3</v>
       </c>
     </row>
     <row r="179">
@@ -2896,13 +2896,13 @@
         <v>06/27</v>
       </c>
       <c r="B179">
-        <v>251.9654545454545</v>
+        <v>251.96545454545458</v>
       </c>
       <c r="C179">
         <v>11</v>
       </c>
       <c r="D179">
-        <v>2771.6199999999994</v>
+        <v>2771.6200000000003</v>
       </c>
     </row>
     <row r="180">
@@ -3311,9 +3311,107 @@
         <v>2140.4</v>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>07/27</v>
+      </c>
+      <c r="B209">
+        <v>198.87142857142857</v>
+      </c>
+      <c r="C209">
+        <v>7</v>
+      </c>
+      <c r="D209">
+        <v>1392.1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>07/28</v>
+      </c>
+      <c r="B210">
+        <v>197.51111111111112</v>
+      </c>
+      <c r="C210">
+        <v>9</v>
+      </c>
+      <c r="D210">
+        <v>1777.6000000000001</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>07/29</v>
+      </c>
+      <c r="B211">
+        <v>218.04444444444445</v>
+      </c>
+      <c r="C211">
+        <v>9</v>
+      </c>
+      <c r="D211">
+        <v>1962.4</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>07/30</v>
+      </c>
+      <c r="B212">
+        <v>242.28571428571428</v>
+      </c>
+      <c r="C212">
+        <v>7</v>
+      </c>
+      <c r="D212">
+        <v>1696</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>07/31</v>
+      </c>
+      <c r="B213">
+        <v>271.21818181818185</v>
+      </c>
+      <c r="C213">
+        <v>11</v>
+      </c>
+      <c r="D213">
+        <v>2983.4</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>08/01</v>
+      </c>
+      <c r="B214">
+        <v>249.6916666666667</v>
+      </c>
+      <c r="C214">
+        <v>12</v>
+      </c>
+      <c r="D214">
+        <v>2996.3</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>08/02</v>
+      </c>
+      <c r="B215">
+        <v>204.25</v>
+      </c>
+      <c r="C215">
+        <v>8</v>
+      </c>
+      <c r="D215">
+        <v>1634</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D208"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D215"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-08-12
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D215"/>
+  <dimension ref="A1:D222"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2392,13 +2392,13 @@
         <v>05/22</v>
       </c>
       <c r="B143">
-        <v>278.49444444444447</v>
+        <v>278.4944444444444</v>
       </c>
       <c r="C143">
         <v>9</v>
       </c>
       <c r="D143">
-        <v>2506.4500000000003</v>
+        <v>2506.45</v>
       </c>
     </row>
     <row r="144">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.2125</v>
+        <v>256.21250000000003</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.5499999999997</v>
+        <v>3074.55</v>
       </c>
     </row>
     <row r="145">
@@ -2504,13 +2504,13 @@
         <v>05/30</v>
       </c>
       <c r="B151">
-        <v>274.58000000000004</v>
+        <v>274.58</v>
       </c>
       <c r="C151">
         <v>5</v>
       </c>
       <c r="D151">
-        <v>1372.9</v>
+        <v>1372.8999999999999</v>
       </c>
     </row>
     <row r="152">
@@ -2672,13 +2672,13 @@
         <v>06/11</v>
       </c>
       <c r="B163">
-        <v>237.04999999999998</v>
+        <v>237.05000000000004</v>
       </c>
       <c r="C163">
         <v>6</v>
       </c>
       <c r="D163">
-        <v>1422.3</v>
+        <v>1422.3000000000002</v>
       </c>
     </row>
     <row r="164">
@@ -2756,13 +2756,13 @@
         <v>06/17</v>
       </c>
       <c r="B169">
-        <v>212.05666666666667</v>
+        <v>212.0566666666667</v>
       </c>
       <c r="C169">
         <v>9</v>
       </c>
       <c r="D169">
-        <v>1908.51</v>
+        <v>1908.5100000000002</v>
       </c>
     </row>
     <row r="170">
@@ -2784,13 +2784,13 @@
         <v>06/19</v>
       </c>
       <c r="B171">
-        <v>274.144</v>
+        <v>274.14399999999995</v>
       </c>
       <c r="C171">
         <v>10</v>
       </c>
       <c r="D171">
-        <v>2741.44</v>
+        <v>2741.4399999999996</v>
       </c>
     </row>
     <row r="172">
@@ -2798,13 +2798,13 @@
         <v>06/20</v>
       </c>
       <c r="B172">
-        <v>300.12333333333333</v>
+        <v>300.1233333333333</v>
       </c>
       <c r="C172">
         <v>9</v>
       </c>
       <c r="D172">
-        <v>2701.11</v>
+        <v>2701.1099999999997</v>
       </c>
     </row>
     <row r="173">
@@ -2812,13 +2812,13 @@
         <v>06/21</v>
       </c>
       <c r="B173">
-        <v>240.55714285714288</v>
+        <v>240.55714285714285</v>
       </c>
       <c r="C173">
         <v>7</v>
       </c>
       <c r="D173">
-        <v>1683.9</v>
+        <v>1683.8999999999999</v>
       </c>
     </row>
     <row r="174">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>257.81111111111113</v>
+        <v>257.8111111111111</v>
       </c>
       <c r="C178">
         <v>9</v>
       </c>
       <c r="D178">
-        <v>2320.3</v>
+        <v>2320.2999999999997</v>
       </c>
     </row>
     <row r="179">
@@ -3078,13 +3078,13 @@
         <v>07/10</v>
       </c>
       <c r="B192">
-        <v>317.1272727272727</v>
+        <v>317.12727272727267</v>
       </c>
       <c r="C192">
         <v>11</v>
       </c>
       <c r="D192">
-        <v>3488.4</v>
+        <v>3488.3999999999996</v>
       </c>
     </row>
     <row r="193">
@@ -3330,13 +3330,13 @@
         <v>07/28</v>
       </c>
       <c r="B210">
-        <v>197.51111111111112</v>
+        <v>197.5111111111111</v>
       </c>
       <c r="C210">
         <v>9</v>
       </c>
       <c r="D210">
-        <v>1777.6000000000001</v>
+        <v>1777.6</v>
       </c>
     </row>
     <row r="211">
@@ -3409,9 +3409,107 @@
         <v>1634</v>
       </c>
     </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>08/03</v>
+      </c>
+      <c r="B216">
+        <v>232.16666666666666</v>
+      </c>
+      <c r="C216">
+        <v>6</v>
+      </c>
+      <c r="D216">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>08/04</v>
+      </c>
+      <c r="B217">
+        <v>219</v>
+      </c>
+      <c r="C217">
+        <v>4</v>
+      </c>
+      <c r="D217">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>08/05</v>
+      </c>
+      <c r="B218">
+        <v>240.898</v>
+      </c>
+      <c r="C218">
+        <v>5</v>
+      </c>
+      <c r="D218">
+        <v>1204.49</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>08/06</v>
+      </c>
+      <c r="B219">
+        <v>260.01666666666665</v>
+      </c>
+      <c r="C219">
+        <v>6</v>
+      </c>
+      <c r="D219">
+        <v>1560.1</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>08/07</v>
+      </c>
+      <c r="B220">
+        <v>286.71666666666664</v>
+      </c>
+      <c r="C220">
+        <v>12</v>
+      </c>
+      <c r="D220">
+        <v>3440.6</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>08/08</v>
+      </c>
+      <c r="B221">
+        <v>271.65833333333336</v>
+      </c>
+      <c r="C221">
+        <v>12</v>
+      </c>
+      <c r="D221">
+        <v>3259.9</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>08/09</v>
+      </c>
+      <c r="B222">
+        <v>324.8333333333333</v>
+      </c>
+      <c r="C222">
+        <v>6</v>
+      </c>
+      <c r="D222">
+        <v>1949</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D215"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D222"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-08-17
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D222"/>
+  <dimension ref="A1:D229"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2392,13 +2392,13 @@
         <v>05/22</v>
       </c>
       <c r="B143">
-        <v>278.4944444444444</v>
+        <v>278.49444444444447</v>
       </c>
       <c r="C143">
         <v>9</v>
       </c>
       <c r="D143">
-        <v>2506.45</v>
+        <v>2506.4500000000003</v>
       </c>
     </row>
     <row r="144">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.21250000000003</v>
+        <v>256.2125</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.55</v>
+        <v>3074.5499999999997</v>
       </c>
     </row>
     <row r="145">
@@ -2700,13 +2700,13 @@
         <v>06/13</v>
       </c>
       <c r="B165">
-        <v>245.7977777777778</v>
+        <v>245.79777777777775</v>
       </c>
       <c r="C165">
         <v>9</v>
       </c>
       <c r="D165">
-        <v>2212.1800000000003</v>
+        <v>2212.18</v>
       </c>
     </row>
     <row r="166">
@@ -2714,13 +2714,13 @@
         <v>06/14</v>
       </c>
       <c r="B166">
-        <v>225.42499999999998</v>
+        <v>225.42500000000004</v>
       </c>
       <c r="C166">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>1352.55</v>
+        <v>1352.5500000000002</v>
       </c>
     </row>
     <row r="167">
@@ -2742,13 +2742,13 @@
         <v>06/16</v>
       </c>
       <c r="B168">
-        <v>199.76999999999998</v>
+        <v>199.77</v>
       </c>
       <c r="C168">
         <v>6</v>
       </c>
       <c r="D168">
-        <v>1198.62</v>
+        <v>1198.6200000000001</v>
       </c>
     </row>
     <row r="169">
@@ -2756,13 +2756,13 @@
         <v>06/17</v>
       </c>
       <c r="B169">
-        <v>212.0566666666667</v>
+        <v>212.05666666666667</v>
       </c>
       <c r="C169">
         <v>9</v>
       </c>
       <c r="D169">
-        <v>1908.5100000000002</v>
+        <v>1908.51</v>
       </c>
     </row>
     <row r="170">
@@ -2784,13 +2784,13 @@
         <v>06/19</v>
       </c>
       <c r="B171">
-        <v>274.14399999999995</v>
+        <v>274.144</v>
       </c>
       <c r="C171">
         <v>10</v>
       </c>
       <c r="D171">
-        <v>2741.4399999999996</v>
+        <v>2741.44</v>
       </c>
     </row>
     <row r="172">
@@ -2812,13 +2812,13 @@
         <v>06/21</v>
       </c>
       <c r="B173">
-        <v>240.55714285714285</v>
+        <v>240.55714285714288</v>
       </c>
       <c r="C173">
         <v>7</v>
       </c>
       <c r="D173">
-        <v>1683.8999999999999</v>
+        <v>1683.9</v>
       </c>
     </row>
     <row r="174">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>257.8111111111111</v>
+        <v>257.81111111111113</v>
       </c>
       <c r="C178">
         <v>9</v>
       </c>
       <c r="D178">
-        <v>2320.2999999999997</v>
+        <v>2320.3</v>
       </c>
     </row>
     <row r="179">
@@ -2896,13 +2896,13 @@
         <v>06/27</v>
       </c>
       <c r="B179">
-        <v>251.96545454545458</v>
+        <v>251.96545454545455</v>
       </c>
       <c r="C179">
         <v>11</v>
       </c>
       <c r="D179">
-        <v>2771.6200000000003</v>
+        <v>2771.62</v>
       </c>
     </row>
     <row r="180">
@@ -3078,13 +3078,13 @@
         <v>07/10</v>
       </c>
       <c r="B192">
-        <v>317.12727272727267</v>
+        <v>317.1272727272727</v>
       </c>
       <c r="C192">
         <v>11</v>
       </c>
       <c r="D192">
-        <v>3488.3999999999996</v>
+        <v>3488.4</v>
       </c>
     </row>
     <row r="193">
@@ -3232,13 +3232,13 @@
         <v>07/21</v>
       </c>
       <c r="B203">
-        <v>169.42249999999999</v>
+        <v>169.4225</v>
       </c>
       <c r="C203">
         <v>4</v>
       </c>
       <c r="D203">
-        <v>677.6899999999999</v>
+        <v>677.69</v>
       </c>
     </row>
     <row r="204">
@@ -3294,7 +3294,7 @@
         <v>11</v>
       </c>
       <c r="D207">
-        <v>2833.38</v>
+        <v>2833.3799999999997</v>
       </c>
     </row>
     <row r="208">
@@ -3330,13 +3330,13 @@
         <v>07/28</v>
       </c>
       <c r="B210">
-        <v>197.5111111111111</v>
+        <v>197.51111111111112</v>
       </c>
       <c r="C210">
         <v>9</v>
       </c>
       <c r="D210">
-        <v>1777.6</v>
+        <v>1777.6000000000001</v>
       </c>
     </row>
     <row r="211">
@@ -3470,13 +3470,13 @@
         <v>08/07</v>
       </c>
       <c r="B220">
-        <v>286.71666666666664</v>
+        <v>266.05</v>
       </c>
       <c r="C220">
         <v>12</v>
       </c>
       <c r="D220">
-        <v>3440.6</v>
+        <v>3192.6</v>
       </c>
     </row>
     <row r="221">
@@ -3484,13 +3484,13 @@
         <v>08/08</v>
       </c>
       <c r="B221">
-        <v>271.65833333333336</v>
+        <v>250.74166666666667</v>
       </c>
       <c r="C221">
         <v>12</v>
       </c>
       <c r="D221">
-        <v>3259.9</v>
+        <v>3008.9</v>
       </c>
     </row>
     <row r="222">
@@ -3498,18 +3498,116 @@
         <v>08/09</v>
       </c>
       <c r="B222">
-        <v>324.8333333333333</v>
+        <v>244.66666666666666</v>
       </c>
       <c r="C222">
         <v>6</v>
       </c>
       <c r="D222">
-        <v>1949</v>
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>08/10</v>
+      </c>
+      <c r="B223">
+        <v>236.66666666666666</v>
+      </c>
+      <c r="C223">
+        <v>3</v>
+      </c>
+      <c r="D223">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>08/11</v>
+      </c>
+      <c r="B224">
+        <v>0</v>
+      </c>
+      <c r="C224">
+        <v>0</v>
+      </c>
+      <c r="D224">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>08/12</v>
+      </c>
+      <c r="B225">
+        <v>0</v>
+      </c>
+      <c r="C225">
+        <v>0</v>
+      </c>
+      <c r="D225">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>08/13</v>
+      </c>
+      <c r="B226">
+        <v>93.5</v>
+      </c>
+      <c r="C226">
+        <v>2</v>
+      </c>
+      <c r="D226">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>08/14</v>
+      </c>
+      <c r="B227">
+        <v>250.86363636363637</v>
+      </c>
+      <c r="C227">
+        <v>11</v>
+      </c>
+      <c r="D227">
+        <v>2759.5</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>08/15</v>
+      </c>
+      <c r="B228">
+        <v>240.29999999999998</v>
+      </c>
+      <c r="C228">
+        <v>11</v>
+      </c>
+      <c r="D228">
+        <v>2643.2999999999997</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>08/16</v>
+      </c>
+      <c r="B229">
+        <v>199.45666666666668</v>
+      </c>
+      <c r="C229">
+        <v>3</v>
+      </c>
+      <c r="D229">
+        <v>598.37</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D222"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D229"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Cloudbeds export from Drive — 2026-08-25
</commit_message>
<xml_diff>
--- a/ok-fc_occupancy_2026ytd.xlsx
+++ b/ok-fc_occupancy_2026ytd.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D229"/>
+  <dimension ref="A1:D236"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1034,13 +1034,13 @@
         <v>02/14</v>
       </c>
       <c r="B46">
-        <v>202.016</v>
+        <v>202.01600000000002</v>
       </c>
       <c r="C46">
         <v>5</v>
       </c>
       <c r="D46">
-        <v>1010.0799999999999</v>
+        <v>1010.08</v>
       </c>
     </row>
     <row r="47">
@@ -2392,13 +2392,13 @@
         <v>05/22</v>
       </c>
       <c r="B143">
-        <v>278.49444444444447</v>
+        <v>278.4944444444444</v>
       </c>
       <c r="C143">
         <v>9</v>
       </c>
       <c r="D143">
-        <v>2506.4500000000003</v>
+        <v>2506.45</v>
       </c>
     </row>
     <row r="144">
@@ -2406,13 +2406,13 @@
         <v>05/23</v>
       </c>
       <c r="B144">
-        <v>256.2125</v>
+        <v>256.21250000000003</v>
       </c>
       <c r="C144">
         <v>12</v>
       </c>
       <c r="D144">
-        <v>3074.5499999999997</v>
+        <v>3074.55</v>
       </c>
     </row>
     <row r="145">
@@ -2426,7 +2426,7 @@
         <v>10</v>
       </c>
       <c r="D145">
-        <v>2962.45</v>
+        <v>2962.4500000000003</v>
       </c>
     </row>
     <row r="146">
@@ -2448,13 +2448,13 @@
         <v>05/26</v>
       </c>
       <c r="B147">
-        <v>190.15555555555554</v>
+        <v>190.15555555555557</v>
       </c>
       <c r="C147">
         <v>9</v>
       </c>
       <c r="D147">
-        <v>1711.3999999999999</v>
+        <v>1711.4</v>
       </c>
     </row>
     <row r="148">
@@ -2742,13 +2742,13 @@
         <v>06/16</v>
       </c>
       <c r="B168">
-        <v>199.77</v>
+        <v>199.76999999999998</v>
       </c>
       <c r="C168">
         <v>6</v>
       </c>
       <c r="D168">
-        <v>1198.6200000000001</v>
+        <v>1198.62</v>
       </c>
     </row>
     <row r="169">
@@ -2784,13 +2784,13 @@
         <v>06/19</v>
       </c>
       <c r="B171">
-        <v>274.144</v>
+        <v>274.14399999999995</v>
       </c>
       <c r="C171">
         <v>10</v>
       </c>
       <c r="D171">
-        <v>2741.44</v>
+        <v>2741.4399999999996</v>
       </c>
     </row>
     <row r="172">
@@ -2798,13 +2798,13 @@
         <v>06/20</v>
       </c>
       <c r="B172">
-        <v>300.1233333333333</v>
+        <v>300.12333333333333</v>
       </c>
       <c r="C172">
         <v>9</v>
       </c>
       <c r="D172">
-        <v>2701.1099999999997</v>
+        <v>2701.11</v>
       </c>
     </row>
     <row r="173">
@@ -2812,13 +2812,13 @@
         <v>06/21</v>
       </c>
       <c r="B173">
-        <v>240.55714285714288</v>
+        <v>240.55714285714285</v>
       </c>
       <c r="C173">
         <v>7</v>
       </c>
       <c r="D173">
-        <v>1683.9</v>
+        <v>1683.8999999999999</v>
       </c>
     </row>
     <row r="174">
@@ -2882,13 +2882,13 @@
         <v>06/26</v>
       </c>
       <c r="B178">
-        <v>257.81111111111113</v>
+        <v>257.8111111111111</v>
       </c>
       <c r="C178">
         <v>9</v>
       </c>
       <c r="D178">
-        <v>2320.3</v>
+        <v>2320.2999999999997</v>
       </c>
     </row>
     <row r="179">
@@ -3232,13 +3232,13 @@
         <v>07/21</v>
       </c>
       <c r="B203">
-        <v>169.4225</v>
+        <v>169.42249999999999</v>
       </c>
       <c r="C203">
         <v>4</v>
       </c>
       <c r="D203">
-        <v>677.69</v>
+        <v>677.6899999999999</v>
       </c>
     </row>
     <row r="204">
@@ -3294,7 +3294,7 @@
         <v>11</v>
       </c>
       <c r="D207">
-        <v>2833.3799999999997</v>
+        <v>2833.38</v>
       </c>
     </row>
     <row r="208">
@@ -3330,13 +3330,13 @@
         <v>07/28</v>
       </c>
       <c r="B210">
-        <v>197.51111111111112</v>
+        <v>197.5111111111111</v>
       </c>
       <c r="C210">
         <v>9</v>
       </c>
       <c r="D210">
-        <v>1777.6000000000001</v>
+        <v>1777.6</v>
       </c>
     </row>
     <row r="211">
@@ -3582,13 +3582,13 @@
         <v>08/15</v>
       </c>
       <c r="B228">
-        <v>240.29999999999998</v>
+        <v>240.3</v>
       </c>
       <c r="C228">
         <v>11</v>
       </c>
       <c r="D228">
-        <v>2643.2999999999997</v>
+        <v>2643.3</v>
       </c>
     </row>
     <row r="229">
@@ -3605,9 +3605,107 @@
         <v>598.37</v>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>08/17</v>
+      </c>
+      <c r="B230">
+        <v>254.5</v>
+      </c>
+      <c r="C230">
+        <v>2</v>
+      </c>
+      <c r="D230">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>08/18</v>
+      </c>
+      <c r="B231">
+        <v>239</v>
+      </c>
+      <c r="C231">
+        <v>1</v>
+      </c>
+      <c r="D231">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>08/19</v>
+      </c>
+      <c r="B232">
+        <v>239</v>
+      </c>
+      <c r="C232">
+        <v>1</v>
+      </c>
+      <c r="D232">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>08/20</v>
+      </c>
+      <c r="B233">
+        <v>0</v>
+      </c>
+      <c r="C233">
+        <v>0</v>
+      </c>
+      <c r="D233">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>08/21</v>
+      </c>
+      <c r="B234">
+        <v>237.72</v>
+      </c>
+      <c r="C234">
+        <v>6</v>
+      </c>
+      <c r="D234">
+        <v>1426.32</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>08/22</v>
+      </c>
+      <c r="B235">
+        <v>242.7033333333333</v>
+      </c>
+      <c r="C235">
+        <v>6</v>
+      </c>
+      <c r="D235">
+        <v>1456.2199999999998</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>08/23</v>
+      </c>
+      <c r="B236">
+        <v>215.55</v>
+      </c>
+      <c r="C236">
+        <v>4</v>
+      </c>
+      <c r="D236">
+        <v>862.2</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D229"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D236"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>